<commit_message>
Regenerate branch functionality spreadsheet
</commit_message>
<xml_diff>
--- a/Docs/Branch_Functionality_Matrix.xlsx
+++ b/Docs/Branch_Functionality_Matrix.xlsx
@@ -12,20 +12,29 @@
       <name val="Aptos"/>
     </font>
   </fonts>
-  <fills count="1">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -43,9 +52,9 @@
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="42" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="5" width="72" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="74" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -66,7 +75,7 @@
       </c>
       <c r="D1" t="inlineStr" s="1">
         <is>
-          <t>codex/experimental-features</t>
+          <t>experimental-features</t>
         </is>
       </c>
       <c r="E1" t="inlineStr" s="1">
@@ -98,7 +107,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Shared stable UI: octopus mark, black canvas, depth, TTV, RunTime, ascent gauge, stopwatch.</t>
+          <t>Octopus mark, black canvas, depth, TTV, RunTime, ascent gauge, stopwatch.</t>
         </is>
       </c>
     </row>
@@ -503,7 +512,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Docs/EXPERIMENTAL_FEATURES.md and Buddy preview only in experimental.</t>
+          <t>EXPERIMENTAL_FEATURES.md and Buddy preview only in experimental.</t>
         </is>
       </c>
     </row>
@@ -530,7 +539,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Lives on branch main-iOS, not in main or codex/experimental-features.</t>
+          <t>Lives on branch main-iOS, not in main or experimental-features.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add iOS experimental branch to matrix
</commit_message>
<xml_diff>
--- a/Docs/Branch_Functionality_Matrix.xlsx
+++ b/Docs/Branch_Functionality_Matrix.xlsx
@@ -133,10 +133,10 @@
 <file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="42" customWidth="1"/>
-    <col min="3" max="5" width="23" customWidth="1"/>
-    <col min="6" max="6" width="76" customWidth="1"/>
+    <col min="3" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="78" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -170,6 +170,11 @@
           <t/>
         </is>
       </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -202,34 +207,44 @@
           <t/>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Branch commits</t>
+          <t>Compared branches</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>main da4541f</t>
+          <t>main</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>experimental-features 3fe5ec4</t>
+          <t>codex/experimental-features</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>main-iOS afcab8e</t>
+          <t>main-iOS</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t/>
+          <t>codex/ios-experimental-features</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -238,27 +253,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t/>
+          <t>Reference commits</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t/>
+          <t>main c3af69b</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t/>
+          <t>watch experimental 3fe5ec4</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t/>
+          <t>main-iOS afcab8e</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t/>
+          <t>iOS experimental 39cfa20</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -266,68 +281,83 @@
           <t/>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr" s="2">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="2">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr" s="2">
+      <c r="B6" t="inlineStr" s="2">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr" s="2">
+      <c r="C6" t="inlineStr" s="2">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr" s="2">
+      <c r="D6" t="inlineStr" s="2">
         <is>
           <t>codex/experimental-features</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr" s="2">
+      <c r="E6" t="inlineStr" s="2">
         <is>
           <t>main-iOS</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr" s="2">
+      <c r="F6" t="inlineStr" s="2">
+        <is>
+          <t>codex/ios-experimental-features</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr" s="2">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Platform</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Apple Watch app</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr" s="3">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr" s="3">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr" s="4">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>watchOS app lives in main and experimental-features.</t>
         </is>
       </c>
     </row>
@@ -339,59 +369,69 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>iPhone companion app</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr" s="4">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr" s="4">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr" s="3">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>iOS companion app lives only in main-iOS.</t>
+          <t>Apple Watch app</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>watchOS app lives in main and Watch experimental.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Watch premium dive-computer look and feel</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr" s="3">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr" s="3">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr" s="4">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Black canvas, thin technical panels, octopus mark, large depth, colored ascent gauge.</t>
+          <t>iPhone companion app</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>iOS app lives in main-iOS and iOS experimental.</t>
         </is>
       </c>
     </row>
@@ -403,59 +443,69 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>iOS companion premium mockup look and feel</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr" s="4">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr" s="4">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr" s="3">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Dark cyan iPhone UI aligned to the supplied iOS mockup.</t>
+          <t>Watch premium dive-computer look and feel</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Black canvas, octopus mark, large depth, technical panels.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Dive Core</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Apple water submersion API scaffold</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr" s="3">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr" s="3">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr" s="4">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Entitlement still pending for production depth data.</t>
+          <t>iOS companion premium dark cyan look and feel</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>iOS companion follows supplied iPhone mockup style.</t>
         </is>
       </c>
     </row>
@@ -467,7 +517,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Current/max/average depth, temperature, runtime, TTV</t>
+          <t>Apple water submersion API scaffold</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="3">
@@ -480,14 +530,19 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr" s="5">
-        <is>
-          <t>Display/reference only</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Core live metrics are watchOS features.</t>
+      <c r="E11" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Entitlement still pending for production depth data.</t>
         </is>
       </c>
     </row>
@@ -499,7 +554,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Manual stopwatch controls</t>
+          <t>Current/max/average depth, temperature, runtime, TTV</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="3">
@@ -512,14 +567,19 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr" s="4">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>START, STOP, RESET on Apple Watch.</t>
+      <c r="E12" t="inlineStr" s="5">
+        <is>
+          <t>Display/reference only</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr" s="5">
+        <is>
+          <t>Display/reference only</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Core live metrics are watchOS runtime features.</t>
         </is>
       </c>
     </row>
@@ -531,7 +591,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ascent-rate gauge</t>
+          <t>Manual stopwatch controls</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="3">
@@ -544,14 +604,19 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr" s="5">
-        <is>
-          <t>Planner/reference only</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Watch live gauge uses green/yellow/red zones.</t>
+      <c r="E13" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>START, STOP, RESET on Apple Watch.</t>
         </is>
       </c>
     </row>
@@ -563,7 +628,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>User-configurable ascent-rate limits</t>
+          <t>Ascent-rate gauge</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="3">
@@ -576,26 +641,31 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr" s="4">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Stored locally via UserDefaults on watchOS.</t>
+      <c r="E14" t="inlineStr" s="5">
+        <is>
+          <t>Planner/reference only</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr" s="5">
+        <is>
+          <t>Planner/reference only</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Watch live gauge uses green/yellow/red zones.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Dive Core</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Compass screen and bearing controls</t>
+          <t>User-configurable ascent-rate limits</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="3">
@@ -613,21 +683,26 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>CoreLocation heading with SET/CLEAR bearing.</t>
+      <c r="F15" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Stored locally on watchOS.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Logging</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Local dive log persistence</t>
+          <t>Compass screen and bearing controls</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="3">
@@ -640,14 +715,19 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr" s="3">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Watch and iOS maintain local log models.</t>
+      <c r="E16" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr" s="5">
+        <is>
+          <t>Buddy companion view only</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>iOS experimental mirrors plausible direction status only.</t>
         </is>
       </c>
     </row>
@@ -659,7 +739,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Dive detail and profile chart</t>
+          <t>Local dive log persistence</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="3">
@@ -677,9 +757,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>iOS has richer companion detail views.</t>
+      <c r="F17" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Watch and iOS maintain local log models.</t>
         </is>
       </c>
     </row>
@@ -691,7 +776,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>GPS entry/exit metadata</t>
+          <t>Dive detail and profile chart</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="3">
@@ -709,21 +794,26 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Watch captures; iOS model displays/exports where available.</t>
+      <c r="F18" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>iOS has richer companion detail views.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Export</t>
+          <t>Logging</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Subsurface CSV export</t>
+          <t>GPS entry/exit metadata</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="3">
@@ -741,21 +831,26 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>CSV export service exists on watch and iOS companion.</t>
+      <c r="F19" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Watch captures; iOS displays/exports where available.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Export</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Bundled user images/checklists screen</t>
+          <t>Subsurface CSV export</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="3">
@@ -768,31 +863,36 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr" s="4">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Watch-only bundled image viewer.</t>
+      <c r="E20" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>CSV export service exists on watch and iOS companion.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Experimental</t>
+          <t>Reference</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Buddy Assist preset messaging</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr" s="4">
-        <is>
-          <t>No</t>
+          <t>Bundled user images/checklists screen</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D21" t="inlineStr" s="3">
@@ -805,21 +905,26 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Must remain isolated from main.</t>
+      <c r="F21" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Watch-only bundled image viewer.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Experimental</t>
+          <t>Experimental Watch</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Buddy Link proximity indicator</t>
+          <t>Buddy Assist preset messaging</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="4">
@@ -837,21 +942,26 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>RSSI ping every 15 seconds with green/yellow/red status.</t>
+      <c r="F22" t="inlineStr" s="5">
+        <is>
+          <t>Companion preparation only</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Actual Buddy message runtime remains Watch experimental.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Experimental</t>
+          <t>Experimental Watch</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Received Buddy message banner and answer flow</t>
+          <t>Buddy Link proximity indicator</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="4">
@@ -869,21 +979,26 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>ANSWER uses the same preset message set.</t>
+      <c r="F23" t="inlineStr" s="5">
+        <is>
+          <t>Companion status only</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Watch experimental uses RSSI ping every 15 seconds.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Experimental</t>
+          <t>Experimental Watch</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Buddy compass plausible direction block</t>
+          <t>Received Buddy message banner and answer flow</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="4">
@@ -901,21 +1016,26 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Heading, shared bearing, last known direction.</t>
+      <c r="F24" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>ANSWER flow is Watch-side runtime.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Experimental Watch</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Secure pre-dive Buddy pairing</t>
+          <t>Buddy compass plausible direction block</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="4">
@@ -933,9 +1053,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Pairing locked during active dive; TRUST requires matching confirmation code.</t>
+      <c r="F25" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>iOS experimental mirrors heading/shared bearing/plausible direction.</t>
         </is>
       </c>
     </row>
@@ -947,7 +1072,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Keychain-backed Buddy authentication material</t>
+          <t>Secure pre-dive Buddy pairing</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="4">
@@ -965,9 +1090,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>SecureBuddyStore stores trusted buddy key in Keychain.</t>
+      <c r="F26" t="inlineStr" s="5">
+        <is>
+          <t>Companion review only</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>iOS experimental shows VERIFY/TRUSTED status, code and fingerprint.</t>
         </is>
       </c>
     </row>
@@ -979,7 +1109,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Authenticated Buddy message envelope</t>
+          <t>Keychain-backed Buddy authentication material</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="4">
@@ -997,21 +1127,26 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>HMAC-SHA256 with session, timestamp, sequence, replay rejection.</t>
+      <c r="F27" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Keychain Buddy runtime remains Watch experimental only.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Frameworks</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CoreBluetooth dependency</t>
+          <t>Authenticated Buddy message envelope</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="4">
@@ -1029,9 +1164,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Only experimental-features has BLE scaffolding.</t>
+      <c r="F28" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>HMAC-SHA256 message envelope remains Watch experimental runtime.</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Security.framework dependency</t>
+          <t>CoreBluetooth dependency</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="4">
@@ -1061,21 +1201,26 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Only experimental-features needs Keychain for Buddy keys.</t>
+      <c r="F29" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>BLE scaffolding exists only in Watch experimental.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>iOS Companion</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Logbook screen</t>
+          <t>Security.framework dependency</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="4">
@@ -1083,31 +1228,36 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr" s="4">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr" s="3">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>iPhone companion logbook UI.</t>
+      <c r="D30" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Only Watch experimental needs Keychain for Buddy keys.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>iOS Companion</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dive analytics screen</t>
+          <t>WatchConnectivity dependency</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="4">
@@ -1125,9 +1275,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Advanced statistics and charts.</t>
+      <c r="F31" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>iOS companion uses WatchConnectivity scaffold.</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1294,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dive planner with Buhlmann ZH-L16C</t>
+          <t>Logbook screen</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="4">
@@ -1157,9 +1312,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Planner branch contains Buhlmann planning services.</t>
+      <c r="F32" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>iPhone companion logbook UI.</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1331,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Gas/MOD/decompression planning UI</t>
+          <t>Dive analytics screen</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="4">
@@ -1189,9 +1349,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Planning model and gas plan views.</t>
+      <c r="F33" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Advanced statistics and charts.</t>
         </is>
       </c>
     </row>
@@ -1203,7 +1368,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>WatchConnectivity sync scaffold</t>
+          <t>Dive planner with Buhlmann ZH-L16C</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="4">
@@ -1221,9 +1386,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>WatchSyncService activates WCSession.</t>
+      <c r="F34" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Planner services live in iOS branches.</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1405,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Cloud backup section</t>
+          <t>Gas/MOD/decompression planning UI</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="4">
@@ -1248,83 +1418,357 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr" s="5">
-        <is>
-          <t>Prepared</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>UI indicates iCloud sync prepared / backup to enable.</t>
+      <c r="E35" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Planning model and gas plan views.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>iOS Companion</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Buddy/BLE excluded from main</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr" s="3">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr" s="6">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr" s="6">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>main has no BuddyAssist/SecureBuddy files and no CoreBluetooth/Security dependencies.</t>
+          <t>Equipment screen</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>iOS companion equipment view.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>iOS Experimental</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Buddy Lab tab</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Premium iOS experimental companion surface.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>iOS Experimental</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Secure pairing review UI</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>VERIFY/TRUSTED, confirmation code, fingerprint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>iOS Experimental</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Buddy Link status UI</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>ONLINE/LOST, signal color, RSSI, ping context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>iOS Experimental</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Preset message preparation UI</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Same message set as Watch experimental, no direct BLE send.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>iOS Experimental</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Watch experimental sync notes</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Documents runtime boundary between iOS companion and Watch BLE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Buddy/BLE excluded from main</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr" s="6">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr" s="6">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr" s="6">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>main has no BuddyAssist/SecureBuddy files and no BLE dependencies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Buddy/BLE runtime excluded from iOS stable</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr" s="6">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr" s="6">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr" s="6">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>main-iOS remains stable companion without Buddy Lab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
         <is>
           <t>Experimental features not production safety systems</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr" s="6">
+      <c r="C44" t="inlineStr" s="6">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr" s="3">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr" s="6">
+      <c r="D44" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr" s="6">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Docs keep Buddy Assist and RSSI proximity marked experimental.</t>
+      <c r="F44" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Docs keep Buddy and RSSI proximity marked experimental.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:F37"/>
+  <autoFilter ref="A6:G44"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh functionality matrix after previews
</commit_message>
<xml_diff>
--- a/Docs/Branch_Functionality_Matrix.xlsx
+++ b/Docs/Branch_Functionality_Matrix.xlsx
@@ -258,7 +258,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>main c3af69b</t>
+          <t>main ccfea3f</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -273,7 +273,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>iOS experimental d726e24</t>
+          <t>iOS experimental 0300730</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1767,8 +1767,45 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>iOS Experimental</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Experimental preview screenshots</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Static premium UI previews stored under Docs/iOS/FeatureScreenshots.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A6:G44"/>
+  <autoFilter ref="A6:G45"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh functionality matrix after readiness check
</commit_message>
<xml_diff>
--- a/Docs/Branch_Functionality_Matrix.xlsx
+++ b/Docs/Branch_Functionality_Matrix.xlsx
@@ -258,12 +258,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>main ccfea3f</t>
+          <t>main a766224</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>watch experimental 9c0ac8e</t>
+          <t>watch experimental 2ac26c8</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">

</xml_diff>

<commit_message>
Refresh matrix for exploration specs
</commit_message>
<xml_diff>
--- a/Docs/Branch_Functionality_Matrix.xlsx
+++ b/Docs/Branch_Functionality_Matrix.xlsx
@@ -184,7 +184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -258,12 +258,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>main a766224</t>
+          <t>main a766224 + matrix 85d227a</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>watch experimental 2ac26c8</t>
+          <t>watch experimental e6b02f7</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -273,7 +273,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>iOS experimental 0300730</t>
+          <t>iOS experimental a2ddbfa</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1804,8 +1804,193 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Experimental Watch</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Pre-water mode selector: Diving / Apnea / Snorkeling</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Implemented only in Watch experimental as ModeSelectionView and ExplorationStore.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Experimental Watch</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Snorkeling runtime, waypoint nav, return-to-entry, GPS markers</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr" s="5">
+        <is>
+          <t>Companion planning only</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Watch runtime UI plus companion route planning support.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Experimental Watch</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Apnea timer, recovery assistant, dive counter, warning layer</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr" s="5">
+        <is>
+          <t>Analytics/planning only</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Watch runtime UI plus iOS analytics companion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>iOS Experimental</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Explore tab: snorkeling map, route, waypoint planner</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Premium iOS companion surface, MapLibre/OpenSeaMap-ready.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>iOS Experimental</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Apnea analytics, readiness, fatigue, recovery, export GPX/CSV</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Implemented in ExplorationCenterView and ExplorationPlanningStore.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A6:G45"/>
+  <autoFilter ref="A6:G50"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh matrix after watch UI check
</commit_message>
<xml_diff>
--- a/Docs/Branch_Functionality_Matrix.xlsx
+++ b/Docs/Branch_Functionality_Matrix.xlsx
@@ -258,12 +258,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>main a766224 + matrix 85d227a</t>
+          <t>main 34db54a</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>watch experimental e6b02f7</t>
+          <t>watch experimental 8d15a93</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">

</xml_diff>

<commit_message>
Refresh matrix for iCloud persistence
</commit_message>
<xml_diff>
--- a/Docs/Branch_Functionality_Matrix.xlsx
+++ b/Docs/Branch_Functionality_Matrix.xlsx
@@ -184,7 +184,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -258,22 +258,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>main 34db54a</t>
+          <t>main de30f24</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>watch experimental 8d15a93</t>
+          <t>watch experimental 75ecbcc</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>main-iOS afcab8e</t>
+          <t>main-iOS dfe8985</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>iOS experimental a2ddbfa</t>
+          <t>iOS experimental 41fc6f5</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1989,8 +1989,156 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Persistence</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>iCloud KVS mirror for Watch dive logs</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Watch logs saved locally and mirrored to iCloud when capability is enabled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Persistence</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>iCloud KVS mirror for Watch ascent/exploration settings</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr" s="5">
+        <is>
+          <t>Ascent only</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr" s="3">
+        <is>
+          <t>Ascent + exploration</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Experimental also mirrors Snorkeling/Apnea state; Buddy keys remain Keychain-only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Persistence</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>iCloud KVS mirror for iOS logbook and planner</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>iOS stores logbook sessions and planner inputs locally plus iCloud mirror.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Persistence</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>iCloud KVS mirror for iOS experimental Buddy/Explore state</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr" s="4">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr" s="3">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Experimental iOS persists Buddy Lab, Explore route, waypoint, warning and sync/export state.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A6:G50"/>
+  <autoFilter ref="A6:G54"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh matrix after GPS capture fix
</commit_message>
<xml_diff>
--- a/Docs/Branch_Functionality_Matrix.xlsx
+++ b/Docs/Branch_Functionality_Matrix.xlsx
@@ -563,12 +563,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>main 2c2d335</t>
+          <t>main 9077699</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>watch experimental cd71cc8</t>
+          <t>watch experimental da1f9b3</t>
         </is>
       </c>
       <c r="D4" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Refresh matrix after GPS finalization fix
</commit_message>
<xml_diff>
--- a/Docs/Branch_Functionality_Matrix.xlsx
+++ b/Docs/Branch_Functionality_Matrix.xlsx
@@ -563,12 +563,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>main 9077699</t>
+          <t>main acbafc5</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>watch experimental da1f9b3</t>
+          <t>watch experimental ff00a92</t>
         </is>
       </c>
       <c r="D4" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Refresh matrix after release readiness fixes
</commit_message>
<xml_diff>
--- a/Docs/Branch_Functionality_Matrix.xlsx
+++ b/Docs/Branch_Functionality_Matrix.xlsx
@@ -517,7 +517,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr"/>
@@ -563,22 +563,22 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>main acbafc5</t>
+          <t>main dc916a3</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>watch experimental ff00a92</t>
+          <t>watch experimental 1ece23f</t>
         </is>
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>main-iOS dfe8985</t>
+          <t>main-iOS 6ad130c</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>iOS experimental 476071a</t>
+          <t>iOS experimental 937b261</t>
         </is>
       </c>
       <c r="F4" s="0" t="inlineStr"/>

</xml_diff>

<commit_message>
Refresh matrix after experimental rebases
</commit_message>
<xml_diff>
--- a/Docs/Branch_Functionality_Matrix.xlsx
+++ b/Docs/Branch_Functionality_Matrix.xlsx
@@ -563,12 +563,12 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>main dc916a3</t>
+          <t>main 83f2857</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>watch experimental 1ece23f</t>
+          <t>watch experimental d2019f7</t>
         </is>
       </c>
       <c r="D4" s="0" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>iOS experimental 937b261</t>
+          <t>iOS experimental f0e6ffb</t>
         </is>
       </c>
       <c r="F4" s="0" t="inlineStr"/>

</xml_diff>

<commit_message>
Refresh matrix after documentation audit
</commit_message>
<xml_diff>
--- a/Docs/Branch_Functionality_Matrix.xlsx
+++ b/Docs/Branch_Functionality_Matrix.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>main 83f2857</t>
+          <t>main 48b81db</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -573,12 +573,12 @@
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>main-iOS 6ad130c</t>
+          <t>main-iOS cb8cbd2</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>iOS experimental f0e6ffb</t>
+          <t>iOS experimental f32fe30</t>
         </is>
       </c>
       <c r="F4" s="0" t="inlineStr"/>

</xml_diff>